<commit_message>
Auto update on 2026-03-06 11:06:23
</commit_message>
<xml_diff>
--- a/jama_exports/kp_data.xlsx
+++ b/jama_exports/kp_data.xlsx
@@ -76,6 +76,9 @@
     <t>Veeramanikandan</t>
   </si>
   <si>
+    <t>Kowsalya</t>
+  </si>
+  <si>
     <t>Jagadeesh</t>
   </si>
   <si>
@@ -95,9 +98,6 @@
   </si>
   <si>
     <t>ARUN KUMAR</t>
-  </si>
-  <si>
-    <t>Kowsalya</t>
   </si>
 </sst>
 </file>
@@ -525,25 +525,25 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="I2">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J2">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="K2">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="L2">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="M2">
-        <v>4.24</v>
+        <v>4.11</v>
       </c>
       <c r="N2">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -563,10 +563,10 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3">
         <v>79</v>
@@ -575,16 +575,16 @@
         <v>5</v>
       </c>
       <c r="J3">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="K3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L3">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="M3">
-        <v>4.9</v>
+        <v>4.15</v>
       </c>
       <c r="N3">
         <v>0.07000000000000001</v>
@@ -613,25 +613,25 @@
         <v>1</v>
       </c>
       <c r="H4">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="I4">
         <v>8</v>
       </c>
       <c r="J4">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="K4">
         <v>9</v>
       </c>
       <c r="L4">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="M4">
-        <v>1.71</v>
+        <v>2.12</v>
       </c>
       <c r="N4">
-        <v>0.38</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -651,7 +651,7 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="G5">
         <v>6</v>
@@ -663,16 +663,16 @@
         <v>0</v>
       </c>
       <c r="J5">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="K5">
         <v>6</v>
       </c>
       <c r="L5">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="M5">
-        <v>3.48</v>
+        <v>3.43</v>
       </c>
       <c r="N5">
         <v>0.08</v>
@@ -695,10 +695,10 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G6">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -707,19 +707,19 @@
         <v>0</v>
       </c>
       <c r="J6">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="K6">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L6">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M6">
-        <v>1.6</v>
+        <v>1.59</v>
       </c>
       <c r="N6">
-        <v>0.62</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -777,37 +777,37 @@
         <v>0</v>
       </c>
       <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>59</v>
+      </c>
+      <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>59</v>
+      </c>
+      <c r="K8">
+        <v>2</v>
+      </c>
+      <c r="L8">
         <v>19</v>
       </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>13</v>
-      </c>
-      <c r="G8">
-        <v>3</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>32</v>
-      </c>
-      <c r="K8">
-        <v>3</v>
-      </c>
-      <c r="L8">
-        <v>16</v>
-      </c>
       <c r="M8">
-        <v>2</v>
+        <v>3.11</v>
       </c>
       <c r="N8">
-        <v>0.09</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -821,16 +821,16 @@
         <v>0</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="F9">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="G9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -839,19 +839,19 @@
         <v>0</v>
       </c>
       <c r="J9">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="K9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L9">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="M9">
-        <v>1.88</v>
+        <v>2.63</v>
       </c>
       <c r="N9">
-        <v>0.16</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -871,10 +871,10 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>98</v>
+        <v>39</v>
       </c>
       <c r="G10">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -883,19 +883,19 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <v>98</v>
+        <v>39</v>
       </c>
       <c r="K10">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="L10">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="M10">
-        <v>4.45</v>
+        <v>1.95</v>
       </c>
       <c r="N10">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -915,10 +915,10 @@
         <v>0</v>
       </c>
       <c r="F11">
-        <v>28</v>
+        <v>103</v>
       </c>
       <c r="G11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -927,19 +927,19 @@
         <v>0</v>
       </c>
       <c r="J11">
-        <v>28</v>
+        <v>103</v>
       </c>
       <c r="K11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="L11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="M11">
-        <v>2.33</v>
+        <v>4.29</v>
       </c>
       <c r="N11">
-        <v>0.46</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -959,10 +959,10 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="G12">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -971,19 +971,19 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="K12">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="L12">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="M12">
-        <v>2.29</v>
+        <v>2.33</v>
       </c>
       <c r="N12">
-        <v>1.21</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -1003,10 +1003,10 @@
         <v>0</v>
       </c>
       <c r="F13">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="G13">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -1015,19 +1015,19 @@
         <v>0</v>
       </c>
       <c r="J13">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="K13">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="L13">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="M13">
-        <v>1.75</v>
+        <v>2.22</v>
       </c>
       <c r="N13">
-        <v>0.14</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -1047,10 +1047,10 @@
         <v>0</v>
       </c>
       <c r="F14">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -1059,19 +1059,19 @@
         <v>0</v>
       </c>
       <c r="J14">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="K14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L14">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="M14">
-        <v>2.75</v>
+        <v>1.56</v>
       </c>
       <c r="N14">
-        <v>0</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -1091,10 +1091,10 @@
         <v>0</v>
       </c>
       <c r="F15">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="G15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -1103,19 +1103,19 @@
         <v>0</v>
       </c>
       <c r="J15">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L15">
         <v>15</v>
       </c>
       <c r="M15">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="N15">
-        <v>0.04</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>